<commit_message>
login dengan set password dan ttd
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -107,6 +107,12 @@
   </x:si>
   <x:si>
     <x:t>BA 022/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 027/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-18</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -798,6 +804,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" spans="1:8">
+      <x:c r="A14" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F14" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G14" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H14" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix: ttd 3 pihak saat unduh
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -125,6 +125,9 @@
   </x:si>
   <x:si>
     <x:t>BA 034/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 035/PPNEG1000/VI/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -946,6 +949,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" spans="1:8">
+      <x:c r="A19" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C19" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D19" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E19" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F19" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G19" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H19" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
feat: search in archieve, pertamina button
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -128,6 +128,12 @@
   </x:si>
   <x:si>
     <x:t>BA 035/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 036/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-20</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -975,6 +981,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" spans="1:8">
+      <x:c r="A20" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C20" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D20" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E20" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F20" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G20" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H20" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
feat: filter archive, export to excel
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -134,6 +134,24 @@
   </x:si>
   <x:si>
     <x:t>2026-06-20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 037/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Peminjaman</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Bucky Barnes</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tony Stark</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-02</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1007,6 +1025,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" spans="1:8">
+      <x:c r="A21" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C21" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D21" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E21" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F21" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="G21" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H21" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
edit layout PJ Sign
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -164,6 +164,9 @@
   </x:si>
   <x:si>
     <x:t>2026-06-26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 043/PPNEG1000/VI/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1141,6 +1144,32 @@
         <x:v>49</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" spans="1:8">
+      <x:c r="A25" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C25" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D25" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E25" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F25" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G25" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H25" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix bug hasil editor tdk muncul di docx yg di-download + fix notif
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -167,6 +167,21 @@
   </x:si>
   <x:si>
     <x:t>BA 043/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 025/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Luthfi Alif Pramudya</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 026/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-23</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-24</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1170,6 +1185,84 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" spans="1:8">
+      <x:c r="A26" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B26" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C26" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D26" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E26" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F26" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G26" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H26" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:8">
+      <x:c r="A27" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B27" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C27" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D27" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E27" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F27" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G27" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H27" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:8">
+      <x:c r="A28" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B28" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C28" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D28" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E28" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F28" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G28" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H28" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
loading di tambah pengguna
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -182,6 +182,12 @@
   </x:si>
   <x:si>
     <x:t>2026-06-24</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 028/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sebastian Vettel</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1263,6 +1269,32 @@
         <x:v>55</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" spans="1:8">
+      <x:c r="A29" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B29" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C29" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D29" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E29" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F29" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G29" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H29" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix grafik persetujuan di dashboard approver
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -191,6 +191,12 @@
   </x:si>
   <x:si>
     <x:t>Kimi Raikkonen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 032/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Gus Fring</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1324,6 +1330,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="31" spans="1:8">
+      <x:c r="A31" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B31" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C31" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D31" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E31" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F31" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G31" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H31" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix canvas ttd mobile
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -197,6 +197,18 @@
   </x:si>
   <x:si>
     <x:t>Gus Fring</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 033/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-27</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1356,6 +1368,58 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" spans="1:8">
+      <x:c r="A32" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B32" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C32" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D32" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E32" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F32" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G32" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H32" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" spans="1:8">
+      <x:c r="A33" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B33" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C33" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D33" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E33" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F33" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G33" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H33" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix tabel header archive
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -209,6 +209,21 @@
   </x:si>
   <x:si>
     <x:t>2026-06-27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 001/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Romi Aprilian Mustafa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 002/PPNEG1000/VI/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1420,6 +1435,58 @@
         <x:v>64</x:v>
       </x:c>
     </x:row>
+    <x:row r="34" spans="1:8">
+      <x:c r="A34" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B34" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C34" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D34" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E34" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F34" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G34" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H34" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" spans="1:8">
+      <x:c r="A35" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B35" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C35" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D35" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E35" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F35" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G35" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H35" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
Edit tombol header preview BA
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -230,6 +230,15 @@
   </x:si>
   <x:si>
     <x:t>2026-07-01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Walter White</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Peter Griffin</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-10</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1519,6 +1528,32 @@
         <x:v>71</x:v>
       </x:c>
     </x:row>
+    <x:row r="37" spans="1:8">
+      <x:c r="A37" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B37" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C37" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D37" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E37" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F37" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G37" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H37" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix flow pengiriman BA, PJ tidak perlu ttd dua kali apabila BA (yang direvisi) di-submit lagi oleh admin gudang barang + tambahan fitur jam pada progress, di mana BA lgsg diteruskan ke approver bila PJ tidak tanda tangan dlm waktu 1x24 jam setelah BA di-submit admin gudang
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -245,6 +245,12 @@
   </x:si>
   <x:si>
     <x:t>BA 008/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 047/PPNEG1000/VI/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-30</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1638,6 +1644,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="41" spans="1:8">
+      <x:c r="A41" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B41" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C41" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D41" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E41" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F41" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G41" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H41" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
update dikit Form BA
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -251,6 +251,12 @@
   </x:si>
   <x:si>
     <x:t>2026-06-30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 018/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Penarikan</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1670,6 +1676,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="42" spans="1:8">
+      <x:c r="A42" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="B42" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C42" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D42" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E42" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F42" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G42" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H42" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
resize field nama PJ dan nama pengguna
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -260,6 +260,9 @@
   </x:si>
   <x:si>
     <x:t>BA 019/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 049/PPNEG1000/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1731,6 +1734,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="44" spans="1:8">
+      <x:c r="A44" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B44" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C44" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D44" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E44" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F44" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G44" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H44" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
pj tdk bisa akses link pada email setelah auto approve
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -275,6 +275,9 @@
   </x:si>
   <x:si>
     <x:t>BA 051/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 052/PPNEG1000/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1824,6 +1827,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="47" spans="1:8">
+      <x:c r="A47" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B47" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C47" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D47" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E47" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F47" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G47" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H47" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix preview in progress menu reviewer and archive bug
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -287,6 +287,9 @@
   </x:si>
   <x:si>
     <x:t>2026-07-03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 009/PPNEG1000/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1914,6 +1917,32 @@
         <x:v>90</x:v>
       </x:c>
     </x:row>
+    <x:row r="50" spans="1:8">
+      <x:c r="A50" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B50" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C50" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D50" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E50" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F50" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G50" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H50" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix: remove PJ rejection email, hide Riwayat action column, and clean up loading UI, Exclude PJ from rejection email notifications; only Admin GB is notified on reject, Remove Silakan hubungi Admin Gudang & Barang text from expired magic link page, Hide Aksi column in Riwayat tab; column only appears in Revisi tab, Strip all text labels from loading overlays, leaving spinner animation only, Restore No. Surat field in reviewer panel with dibuat otomatis saat anda menyetujui, Replace dynamic DasarAlokasi label with static No. Tiket My SSC in document summary
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -290,6 +290,9 @@
   </x:si>
   <x:si>
     <x:t>BA 009/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 011/PPNEG1000/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1943,6 +1946,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="51" spans="1:8">
+      <x:c r="A51" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B51" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C51" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D51" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E51" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F51" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G51" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H51" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
Update alur Approval dari Admin ke Reviewer ke PJ
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -293,6 +293,18 @@
   </x:si>
   <x:si>
     <x:t>BA 024/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 027/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 028/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 029/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 030/PPNEG1000/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1972,6 +1984,110 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="52" spans="1:8">
+      <x:c r="A52" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B52" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C52" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D52" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E52" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F52" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G52" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H52" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" spans="1:8">
+      <x:c r="A53" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B53" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C53" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D53" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E53" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F53" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G53" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H53" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" spans="1:8">
+      <x:c r="A54" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B54" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C54" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D54" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E54" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F54" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G54" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H54" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" spans="1:8">
+      <x:c r="A55" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B55" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C55" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D55" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E55" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F55" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G55" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H55" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
update auto approval real time + stempel, logo SIMBA di login & dashboard, fix error submit
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -311,6 +311,12 @@
   </x:si>
   <x:si>
     <x:t>BA 032/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 003/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA 004/PPNEG1000/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2146,6 +2152,58 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="58" spans="1:8">
+      <x:c r="A58" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B58" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C58" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D58" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E58" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F58" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G58" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H58" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" spans="1:8">
+      <x:c r="A59" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B59" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C59" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D59" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E59" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F59" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G59" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H59" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix import excel bug
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -323,6 +323,12 @@
   </x:si>
   <x:si>
     <x:t>BA-016/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-001/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-05</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2262,6 +2268,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="62" spans="1:8">
+      <x:c r="A62" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="B62" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C62" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D62" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E62" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F62" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G62" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H62" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix peminjaman popout layout in dashboard
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -329,6 +329,15 @@
   </x:si>
   <x:si>
     <x:t>2026-07-05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-002/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-09</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2294,6 +2303,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="63" spans="1:8">
+      <x:c r="A63" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B63" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C63" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D63" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E63" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F63" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G63" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H63" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
Add cancel BA submission Feature, Add SignalR for all menu
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -320,6 +320,15 @@
   </x:si>
   <x:si>
     <x:t>BA 005/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-033/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-034/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-08</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2233,6 +2242,58 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="61" spans="1:8">
+      <x:c r="A61" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B61" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C61" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D61" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E61" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F61" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G61" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H61" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" spans="1:8">
+      <x:c r="A62" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="B62" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C62" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D62" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E62" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F62" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G62" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H62" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
add delete ba lainnya in archive menu
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -329,6 +329,12 @@
   </x:si>
   <x:si>
     <x:t>2026-07-08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-001/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-12</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2294,6 +2300,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="63" spans="1:8">
+      <x:c r="A63" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B63" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C63" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D63" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E63" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F63" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G63" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H63" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix ubah ttd in profile menu bug
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -335,6 +335,21 @@
   </x:si>
   <x:si>
     <x:t>2026-07-12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-005/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-006/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-007/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-008/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BA-002/PPNEG1000/2026-S0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2326,6 +2341,162 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="64" spans="1:8">
+      <x:c r="A64" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B64" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C64" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D64" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E64" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F64" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G64" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H64" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" spans="1:8">
+      <x:c r="A65" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="B65" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C65" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D65" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E65" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F65" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G65" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H65" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" spans="1:8">
+      <x:c r="A66" s="0" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="B66" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C66" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D66" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E66" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F66" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G66" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H66" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" spans="1:8">
+      <x:c r="A67" s="0" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="B67" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C67" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D67" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E67" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F67" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G67" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H67" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" spans="1:8">
+      <x:c r="A68" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B68" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C68" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D68" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E68" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F68" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G68" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H68" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" spans="1:8">
+      <x:c r="A69" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="B69" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C69" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D69" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E69" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F69" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G69" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H69" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix logic numbering BA
</commit_message>
<xml_diff>
--- a/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
+++ b/SistemBeritaAcara.Web/data/ArsipBeritaAcara.xlsx
@@ -350,6 +350,9 @@
   </x:si>
   <x:si>
     <x:t>BA-002/PPNEG1000/2026-S0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-13</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2497,6 +2500,32 @@
         <x:v>15</x:v>
       </x:c>
     </x:row>
+    <x:row r="70" spans="1:8">
+      <x:c r="A70" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B70" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="C70" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D70" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E70" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F70" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G70" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H70" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>